<commit_message>
v6.2: update maternity pants to XL 4x3 (order 3316978813071005461) & sync Oct 25 delivery statuses
</commit_message>
<xml_diff>
--- a/BB已购清单与选品全表_20261024.xlsx
+++ b/BB已购清单与选品全表_20261024.xlsx
@@ -667,7 +667,7 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>已付清</t>
+          <t>已签收·韵达·3栋乙3号丰巢柜</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>已付清</t>
+          <t>已签收·圆通·甲单元丰巢柜</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -805,7 +805,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>卖家已发货·中通</t>
+          <t>已签收·中通·家门口签收</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -874,7 +874,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>已付清</t>
+          <t>已签收·中通·3栋乙1号丰巢柜</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
@@ -1221,7 +1221,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>已付清</t>
+          <t>已签收·中通·3栋乙1号丰巢柜</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
@@ -2256,7 +2256,7 @@
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>已付清</t>
+          <t>已签收·申通·3栋乙3号丰巢柜</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
@@ -2670,7 +2670,7 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>已付清</t>
+          <t>已签收·韵达·3栋乙3号丰巢柜</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>已付清</t>
+          <t>已签收·家门口签收</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr">
@@ -2877,7 +2877,7 @@
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>已付清</t>
+          <t>已签收·家门口签收</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr">
@@ -2912,27 +2912,27 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>嫚熙安睡裤 M-L 4条装（共8条）</t>
+          <t>嫚熙私处冲洗器 抗菌款</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>嫚熙安睡裤 / EMXEE嫚熙母婴用品旗舰店</t>
+          <t>嫚熙私处冲洗器 / EMXEE嫚熙母婴用品旗舰店</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>嫚熙安睡裤 M-L 4条装（共8条）</t>
+          <t>嫚熙私处冲洗器 抗菌款</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>×2</t>
+          <t>×1</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr"/>
       <c r="H36" s="2" t="n">
-        <v>25.97</v>
+        <v>28.68</v>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
@@ -2946,7 +2946,7 @@
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>已付清</t>
+          <t>已签收·中通·丰巢柜</t>
         </is>
       </c>
       <c r="L36" s="2" t="inlineStr">
@@ -2956,12 +2956,12 @@
       </c>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>已加购物车，未付款；大牌官方店/销量高</t>
+          <t>推荐</t>
         </is>
       </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>大牌官方店替换小牌子（10-20）；商品 1077220832978</t>
+          <t>大牌官方旗舰店、口碑稳、性价比合适，按待产包清单必需</t>
         </is>
       </c>
       <c r="O36" s="2" t="inlineStr">
@@ -2981,17 +2981,17 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>嫚熙私处冲洗器 抗菌款</t>
+          <t>舒客密泡月子牙刷 2支装 粉蓝</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>嫚熙私处冲洗器 / EMXEE嫚熙母婴用品旗舰店</t>
+          <t>舒客密泡月子牙刷 / 舒客官方旗舰店</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>嫚熙私处冲洗器 抗菌款</t>
+          <t>舒客密泡月子牙刷 2支装 粉蓝</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -3001,11 +3001,11 @@
       </c>
       <c r="G37" s="2" t="inlineStr"/>
       <c r="H37" s="2" t="n">
-        <v>28.68</v>
+        <v>17.35</v>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>3316545230023689060</t>
+          <t>3316545230023734252</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
@@ -3015,7 +3015,7 @@
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>已付清</t>
+          <t>已签收·申通·3栋乙3号丰巢柜</t>
         </is>
       </c>
       <c r="L37" s="2" t="inlineStr">
@@ -3050,17 +3050,17 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>舒客密泡月子牙刷 2支装 粉蓝</t>
+          <t>茶花一次性弯头吸管 200支</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>舒客密泡月子牙刷 / 舒客官方旗舰店</t>
+          <t>茶花一次性弯头吸管 / 茶花官方旗舰店</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>舒客密泡月子牙刷 2支装 粉蓝</t>
+          <t>茶花一次性弯头吸管 200支</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -3070,11 +3070,11 @@
       </c>
       <c r="G38" s="2" t="inlineStr"/>
       <c r="H38" s="2" t="n">
-        <v>17.35</v>
+        <v>8.609999999999999</v>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>3316545230023734252</t>
+          <t>3316545230023751898</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -3094,7 +3094,7 @@
       </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>推荐</t>
+          <t>—</t>
         </is>
       </c>
       <c r="N38" s="2" t="inlineStr">
@@ -3114,22 +3114,22 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>妈妈用品</t>
+          <t>宝宝喂养</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>茶花一次性弯头吸管 200支</t>
+          <t>英氏奶瓶刷 6合1 硅胶套组</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>茶花一次性弯头吸管 / 茶花官方旗舰店</t>
+          <t>英氏奶瓶刷 / YEEHOOKIDS母婴旗舰店</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>茶花一次性弯头吸管 200支</t>
+          <t>英氏奶瓶刷 6合1 硅胶套组</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -3139,11 +3139,11 @@
       </c>
       <c r="G39" s="2" t="inlineStr"/>
       <c r="H39" s="2" t="n">
-        <v>8.609999999999999</v>
+        <v>32</v>
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>3316545230023751898</t>
+          <t>3316545230023761080</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
@@ -3158,12 +3158,12 @@
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>朋友清单未单列（同类品按需）</t>
+          <t>英式硅胶便携奶瓶刷</t>
         </is>
       </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>未核查</t>
         </is>
       </c>
       <c r="N39" s="2" t="inlineStr">
@@ -3183,22 +3183,22 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>宝宝喂养</t>
+          <t>妈妈用品</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>英氏奶瓶刷 6合1 硅胶套组</t>
+          <t>开丽会阴冷敷贴 体验装2盒</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>英氏奶瓶刷 / YEEHOOKIDS母婴旗舰店</t>
+          <t>开丽会阴冷敷贴 / 开丽旗舰店</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>英氏奶瓶刷 6合1 硅胶套组</t>
+          <t>开丽会阴冷敷贴 体验装2盒</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="G40" s="2" t="inlineStr"/>
       <c r="H40" s="2" t="n">
-        <v>32</v>
+        <v>17.08</v>
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>3316545230023761080</t>
+          <t>3316545230023770262</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -3227,12 +3227,12 @@
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>英式硅胶便携奶瓶刷</t>
+          <t>朋友说医院很贵，提前备（品牌未指定）</t>
         </is>
       </c>
       <c r="M40" s="2" t="inlineStr">
         <is>
-          <t>未核查</t>
+          <t>推荐</t>
         </is>
       </c>
       <c r="N40" s="2" t="inlineStr">
@@ -3252,22 +3252,22 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>妈妈用品</t>
+          <t>纸品纸尿裤</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>开丽会阴冷敷贴 体验装2盒</t>
+          <t>babycare 金山茶 NB 3片试用装</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>开丽会阴冷敷贴 / 开丽旗舰店</t>
+          <t>babycare / bcbabycare纸尿裤旗舰店</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>开丽会阴冷敷贴 体验装2盒</t>
+          <t>babycare 金山茶 NB 3片试用装</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -3277,11 +3277,11 @@
       </c>
       <c r="G41" s="2" t="inlineStr"/>
       <c r="H41" s="2" t="n">
-        <v>17.08</v>
+        <v>4.25</v>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>3316545230023770262</t>
+          <t>3316545230023807089</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
@@ -3296,12 +3296,12 @@
       </c>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>朋友说医院很贵，提前备（品牌未指定）</t>
+          <t>朋友清单未单列（同类品按需）</t>
         </is>
       </c>
       <c r="M41" s="2" t="inlineStr">
         <is>
-          <t>推荐</t>
+          <t>慎重：红屁股/异味投诉</t>
         </is>
       </c>
       <c r="N41" s="2" t="inlineStr">
@@ -3321,22 +3321,22 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>纸品纸尿裤</t>
+          <t>妈妈用品</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>babycare 金山茶 NB 3片试用装</t>
+          <t>十月结晶六合一哺乳枕 2.0 香槟黄</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>babycare / bcbabycare纸尿裤旗舰店</t>
+          <t>十月结晶六合一哺乳枕 / 十月结晶婴童用品旗舰店</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>babycare 金山茶 NB 3片试用装</t>
+          <t>十月结晶六合一哺乳枕 2.0 香槟黄</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -3346,11 +3346,11 @@
       </c>
       <c r="G42" s="2" t="inlineStr"/>
       <c r="H42" s="2" t="n">
-        <v>4.25</v>
+        <v>95</v>
       </c>
       <c r="I42" s="2" t="inlineStr">
         <is>
-          <t>3316545230023807089</t>
+          <t>3316545230023816271</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>已付清</t>
+          <t>已签收·极兔·家门口签收</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr">
@@ -3370,7 +3370,7 @@
       </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>慎重：红屁股/异味投诉</t>
+          <t>可以买但注意：偏矮，可垫毛巾；非必需</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr">
@@ -3390,36 +3390,36 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>妈妈用品</t>
+          <t>宝宝洗护</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>十月结晶六合一哺乳枕 2.0 香槟黄</t>
+          <t>嫚熙纱布浴巾 甜心喵喵 115×115</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>十月结晶六合一哺乳枕 / 十月结晶婴童用品旗舰店</t>
+          <t>嫚熙纱布浴巾 / 嫚熙儿童旗舰店</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>十月结晶六合一哺乳枕 2.0 香槟黄</t>
+          <t>嫚熙纱布浴巾 甜心喵喵 115×115</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>×1</t>
+          <t>×2</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr"/>
       <c r="H43" s="2" t="n">
-        <v>95</v>
+        <v>174.14</v>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>3316545230023816271</t>
+          <t>3316545230023825453</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
@@ -3429,7 +3429,7 @@
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>卖家已发货·极兔</t>
+          <t>已签收·中通·3栋乙1号丰巢柜</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr">
@@ -3439,7 +3439,7 @@
       </c>
       <c r="M43" s="2" t="inlineStr">
         <is>
-          <t>可以买但注意：偏矮，可垫毛巾；非必需</t>
+          <t>可以买但注意：信息少，先洗后用</t>
         </is>
       </c>
       <c r="N43" s="2" t="inlineStr">
@@ -3459,36 +3459,36 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>宝宝洗护</t>
+          <t>宝宝衣物</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>嫚熙纱布浴巾 甜心喵喵 115×115</t>
+          <t>全棉时代拍嗝巾 春日庄园</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>嫚熙纱布浴巾 / 嫚熙儿童旗舰店</t>
+          <t>全棉时代拍嗝巾 / 全棉时代官方旗舰店</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>嫚熙纱布浴巾 甜心喵喵 115×115</t>
+          <t>全棉时代拍嗝巾 春日庄园</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>×2</t>
+          <t>×1</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr"/>
       <c r="H44" s="2" t="n">
-        <v>174.14</v>
+        <v>57.13</v>
       </c>
       <c r="I44" s="2" t="inlineStr">
         <is>
-          <t>3316545230023825453</t>
+          <t>3316545230023843099</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
@@ -3508,12 +3508,12 @@
       </c>
       <c r="M44" s="2" t="inlineStr">
         <is>
-          <t>可以买但注意：信息少，先洗后用</t>
+          <t>已加购物车，未付款；大牌官方店/销量高</t>
         </is>
       </c>
       <c r="N44" s="2" t="inlineStr">
         <is>
-          <t>大牌官方旗舰店、口碑稳、性价比合适，按待产包清单必需</t>
+          <t>大牌官方店替换小牌子（10-20）；商品 713395444860</t>
         </is>
       </c>
       <c r="O44" s="2" t="inlineStr">
@@ -3533,17 +3533,17 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>全棉时代拍嗝巾 春日庄园</t>
+          <t>全棉时代抱被 春日庄园 90×90</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>全棉时代拍嗝巾 / 全棉时代官方旗舰店</t>
+          <t>全棉时代抱被 / 全棉时代官方旗舰店</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>全棉时代拍嗝巾 春日庄园</t>
+          <t>全棉时代抱被 春日庄园 90×90</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -3553,11 +3553,11 @@
       </c>
       <c r="G45" s="2" t="inlineStr"/>
       <c r="H45" s="2" t="n">
-        <v>57.13</v>
+        <v>121.15</v>
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>3316545230023843099</t>
+          <t>3316545230023852281</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
@@ -3577,12 +3577,12 @@
       </c>
       <c r="M45" s="2" t="inlineStr">
         <is>
-          <t>已加购物车，未付款；大牌官方店/销量高</t>
+          <t>3月17日预产期，不选寒冬加厚</t>
         </is>
       </c>
       <c r="N45" s="2" t="inlineStr">
         <is>
-          <t>大牌官方店替换小牌子（10-20）；商品 713395444860</t>
+          <t>大牌官方旗舰店、口碑稳、性价比合适，按待产包清单必需</t>
         </is>
       </c>
       <c r="O45" s="2" t="inlineStr">
@@ -3602,17 +3602,17 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>全棉时代抱被 春日庄园 90×90</t>
+          <t>全棉时代纱布口水巾方巾 快乐河马 25×25</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>全棉时代抱被 / 全棉时代官方旗舰店</t>
+          <t>全棉时代纱布口水巾方巾 / 全棉时代官方旗舰店</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>全棉时代抱被 春日庄园 90×90</t>
+          <t>全棉时代纱布口水巾方巾 快乐河马 25×25</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -3622,7 +3622,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr"/>
       <c r="H46" s="2" t="n">
-        <v>121.15</v>
+        <v>57.88</v>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
@@ -3646,12 +3646,12 @@
       </c>
       <c r="M46" s="2" t="inlineStr">
         <is>
-          <t>3月17日预产期，不选寒冬加厚</t>
+          <t>已加购物车，未付款；大牌官方店/销量高</t>
         </is>
       </c>
       <c r="N46" s="2" t="inlineStr">
         <is>
-          <t>大牌官方旗舰店、口碑稳、性价比合适，按待产包清单必需</t>
+          <t>大牌官方店替换小牌子（10-20）；商品 809465999047</t>
         </is>
       </c>
       <c r="O46" s="2" t="inlineStr">
@@ -3671,17 +3671,17 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>全棉时代纱布口水巾方巾 快乐河马 25×25</t>
+          <t>全棉时代婴儿胎帽 暖纱黄 0-3月（第1顶）</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>全棉时代纱布口水巾方巾 / 全棉时代官方旗舰店</t>
+          <t>全棉时代婴儿胎帽 / 全棉时代官方旗舰店</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>全棉时代纱布口水巾方巾 快乐河马 25×25</t>
+          <t>全棉时代婴儿胎帽 暖纱黄 0-3月（第1顶）</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -3691,7 +3691,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr"/>
       <c r="H47" s="2" t="n">
-        <v>57.88</v>
+        <v>65.34</v>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
@@ -3715,12 +3715,12 @@
       </c>
       <c r="M47" s="2" t="inlineStr">
         <is>
-          <t>已加购物车，未付款；大牌官方店/销量高</t>
+          <t>全棉时代官方旗舰店官方店正品；销量与店铺评分高，未见集中差评</t>
         </is>
       </c>
       <c r="N47" s="2" t="inlineStr">
         <is>
-          <t>大牌官方店替换小牌子（10-20）；商品 809465999047</t>
+          <t>大牌官方旗舰店、口碑稳、性价比合适，按待产包清单必需</t>
         </is>
       </c>
       <c r="O47" s="2" t="inlineStr">
@@ -3740,17 +3740,17 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>全棉时代婴儿胎帽 暖纱黄 0-3月（第1顶）</t>
+          <t>全棉时代婴儿袜 蔚蓝+白+天蓝 0-3月 3双</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>全棉时代婴儿胎帽 / 全棉时代官方旗舰店</t>
+          <t>全棉时代婴儿袜 / 全棉时代官方旗舰店</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>全棉时代婴儿胎帽 暖纱黄 0-3月（第1顶）</t>
+          <t>全棉时代婴儿袜 蔚蓝+白+天蓝 0-3月 3双</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -3760,7 +3760,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr"/>
       <c r="H48" s="2" t="n">
-        <v>65.34</v>
+        <v>40.57</v>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
@@ -3779,17 +3779,17 @@
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>朋友清单未单列（同类品按需）</t>
+          <t>全棉时代 新生儿袜 10-12cm</t>
         </is>
       </c>
       <c r="M48" s="2" t="inlineStr">
         <is>
-          <t>全棉时代官方旗舰店官方店正品；销量与店铺评分高，未见集中差评</t>
+          <t>替换旧 10-12cm 款；新生儿更贴合</t>
         </is>
       </c>
       <c r="N48" s="2" t="inlineStr">
         <is>
-          <t>大牌官方旗舰店、口碑稳、性价比合适，按待产包清单必需</t>
+          <t>商品 930676917108 sku 5981605126182；换 0-3月中筒三色装</t>
         </is>
       </c>
       <c r="O48" s="2" t="inlineStr">
@@ -3804,22 +3804,22 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>宝宝衣物</t>
+          <t>宝宝喂养</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>全棉时代婴儿袜 蔚蓝+白+天蓝 0-3月 3双</t>
+          <t>苏泊尔恒温水壶 4代全玻璃</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>全棉时代婴儿袜 / 全棉时代官方旗舰店</t>
+          <t>苏泊尔恒温水壶 / supor苏泊尔母婴旗舰店</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>全棉时代婴儿袜 蔚蓝+白+天蓝 0-3月 3双</t>
+          <t>苏泊尔恒温水壶 4代全玻璃</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -3829,11 +3829,11 @@
       </c>
       <c r="G49" s="2" t="inlineStr"/>
       <c r="H49" s="2" t="n">
-        <v>40.57</v>
+        <v>216.55</v>
       </c>
       <c r="I49" s="2" t="inlineStr">
         <is>
-          <t>3316545230023852281</t>
+          <t>3316545230023005461</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
@@ -3843,22 +3843,22 @@
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>已付清</t>
+          <t>已签收·圆通·3栋乙2号丰巢柜</t>
         </is>
       </c>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>全棉时代 新生儿袜 10-12cm</t>
+          <t>小白熊 全玻璃恒温壶 ¥324</t>
         </is>
       </c>
       <c r="M49" s="2" t="inlineStr">
         <is>
-          <t>替换旧 10-12cm 款；新生儿更贴合</t>
+          <t>国补单付；全玻璃巢式底座；到手配温度计抽测</t>
         </is>
       </c>
       <c r="N49" s="2" t="inlineStr">
         <is>
-          <t>商品 930676917108 sku 5981605126182；换 0-3月中筒三色装</t>
+          <t>国补单独结算；勿与大单混结以免丢国补；用户改苏泊尔4代全玻璃巢式底座，国补单付约¥214</t>
         </is>
       </c>
       <c r="O49" s="2" t="inlineStr">
@@ -3873,22 +3873,22 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>宝宝喂养</t>
+          <t>妈妈用品</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>苏泊尔恒温水壶 4代全玻璃</t>
+          <t>熊猫布布双边电动吸奶器 Plus</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>苏泊尔恒温水壶 / supor苏泊尔母婴旗舰店</t>
+          <t>熊猫布布双边电动吸奶器 / 熊猫布布旗舰店</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>苏泊尔恒温水壶 4代全玻璃</t>
+          <t>熊猫布布双边电动吸奶器 Plus</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -3898,11 +3898,11 @@
       </c>
       <c r="G50" s="2" t="inlineStr"/>
       <c r="H50" s="2" t="n">
-        <v>216.55</v>
+        <v>1414.24</v>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>3316545230023005461</t>
+          <t>3316545230023032289</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -3917,17 +3917,17 @@
       </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>小白熊 全玻璃恒温壶 ¥324</t>
+          <t>美德乐 致韵Plus</t>
         </is>
       </c>
       <c r="M50" s="2" t="inlineStr">
         <is>
-          <t>国补单付；全玻璃巢式底座；到手配温度计抽测</t>
+          <t>已选定；待加购/问客服延期发货与试用起算；退换期内密集试用；先量乳头选喇叭罩</t>
         </is>
       </c>
       <c r="N50" s="2" t="inlineStr">
         <is>
-          <t>国补单独结算；勿与大单混结以免丢国补；用户改苏泊尔4代全玻璃巢式底座，国补单付约¥214</t>
+          <t>用户选定熊猫布布 Plus（替换美德乐致韵Plus）；客服确认延期发货/试用后再付；用户改回朋友推荐款；待客服确认延期发货与试用起算</t>
         </is>
       </c>
       <c r="O50" s="2" t="inlineStr">
@@ -3942,22 +3942,22 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>妈妈用品</t>
+          <t>宝宝衣物</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>熊猫布布双边电动吸奶器 Plus</t>
+          <t>Baby love 连体衣 星月守护 52cm</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>熊猫布布双边电动吸奶器 / 熊猫布布旗舰店</t>
+          <t>Baby / babylove旗舰店</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>熊猫布布双边电动吸奶器 Plus</t>
+          <t>Baby love 连体衣 星月守护 52cm</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -3967,11 +3967,11 @@
       </c>
       <c r="G51" s="2" t="inlineStr"/>
       <c r="H51" s="2" t="n">
-        <v>1414.24</v>
+        <v>49.56</v>
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>3316545230023032289</t>
+          <t>3316545230023041471</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr">
@@ -3981,22 +3981,22 @@
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>已付清</t>
+          <t>已签收·申通·3栋乙3号丰巢柜</t>
         </is>
       </c>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>美德乐 致韵Plus</t>
+          <t>全棉时代/英氏/babycare/嫚熙 大牌连体衣</t>
         </is>
       </c>
       <c r="M51" s="2" t="inlineStr">
         <is>
-          <t>已选定；待加购/问客服延期发货与试用起算；退换期内密集试用；先量乳头选喇叭罩</t>
+          <t>母婴A类即可；朋友张月推荐；性别中性奶白；先洗后穿</t>
         </is>
       </c>
       <c r="N51" s="2" t="inlineStr">
         <is>
-          <t>用户选定熊猫布布 Plus（替换美德乐致韵Plus）；客服确认延期发货/试用后再付；用户改回朋友推荐款；待客服确认延期发货与试用起算</t>
+          <t>52码奶白缺货故不下；59×3；进店核对A类/系带；半个月就穿不下，改朋友推荐性价比店</t>
         </is>
       </c>
       <c r="O51" s="2" t="inlineStr">
@@ -4016,7 +4016,7 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Baby love 连体衣 星月守护 52cm</t>
+          <t>Baby love 连体衣 奶白 59cm</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -4026,17 +4026,17 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Baby love 连体衣 星月守护 52cm</t>
+          <t>Baby love 连体衣 奶白 59cm</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>×1</t>
+          <t>×3</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr"/>
       <c r="H52" s="2" t="n">
-        <v>49.56</v>
+        <v>187.79</v>
       </c>
       <c r="I52" s="2" t="inlineStr">
         <is>
@@ -4050,7 +4050,7 @@
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>已付清</t>
+          <t>已签收·申通·3栋乙3号丰巢柜</t>
         </is>
       </c>
       <c r="L52" s="2" t="inlineStr">
@@ -4085,31 +4085,31 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Baby love 连体衣 奶白 59cm</t>
+          <t>娃丽比连体衣 萌熊-N8 52cm</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Baby / babylove旗舰店</t>
+          <t>娃丽比连体衣 / 娃丽比母婴旗舰店</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Baby love 连体衣 奶白 59cm</t>
+          <t>娃丽比连体衣 萌熊-N8 52cm</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>×3</t>
+          <t>×1</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr"/>
       <c r="H53" s="2" t="n">
-        <v>187.79</v>
+        <v>66.59</v>
       </c>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>3316545230023041471</t>
+          <t>3316545230023087480</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr">
@@ -4119,22 +4119,22 @@
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>已付清</t>
+          <t>卖家已发货·申通</t>
         </is>
       </c>
       <c r="L53" s="2" t="inlineStr">
         <is>
-          <t>全棉时代/英氏/babycare/嫚熙 大牌连体衣</t>
+          <t>大牌52码连体衣</t>
         </is>
       </c>
       <c r="M53" s="2" t="inlineStr">
         <is>
-          <t>母婴A类即可；朋友张月推荐；性别中性奶白；先洗后穿</t>
+          <t>母婴A类；朋友张月推荐；52合计仅此1件（Baby love 52奶白OOS）；先洗后穿</t>
         </is>
       </c>
       <c r="N53" s="2" t="inlineStr">
         <is>
-          <t>52码奶白缺货故不下；59×3；进店核对A类/系带；半个月就穿不下，改朋友推荐性价比店</t>
+          <t>进店选萌熊52；要孕妈有礼券；朋友推荐娃丽比≈¥70</t>
         </is>
       </c>
       <c r="O53" s="2" t="inlineStr">
@@ -4154,7 +4154,7 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>娃丽比连体衣 萌熊-N8 52cm</t>
+          <t>娃丽比连体衣 萌熊-N8 59cm</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -4164,17 +4164,17 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>娃丽比连体衣 萌熊-N8 52cm</t>
+          <t>娃丽比连体衣 萌熊-N8 59cm</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>×1</t>
+          <t>×3</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr"/>
       <c r="H54" s="2" t="n">
-        <v>66.59</v>
+        <v>199.76</v>
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
@@ -4193,17 +4193,17 @@
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>大牌52码连体衣</t>
+          <t>大牌59码连体衣</t>
         </is>
       </c>
       <c r="M54" s="2" t="inlineStr">
         <is>
-          <t>母婴A类；朋友张月推荐；52合计仅此1件（Baby love 52奶白OOS）；先洗后穿</t>
+          <t>母婴A类；朋友张月推荐；性别中性；先洗后穿</t>
         </is>
       </c>
       <c r="N54" s="2" t="inlineStr">
         <is>
-          <t>进店选萌熊52；要孕妈有礼券；朋友推荐娃丽比≈¥70</t>
+          <t>59合计：Baby love×3 + 娃丽比×3 = 6件；朋友推荐娃丽比≈¥70</t>
         </is>
       </c>
       <c r="O54" s="2" t="inlineStr">
@@ -4218,61 +4218,63 @@
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>宝宝衣物</t>
+          <t>妈妈用品</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>娃丽比连体衣 萌熊-N8 59cm</t>
+          <t>嫚熙安睡裤 XL码 4条×3包（共12条）</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>娃丽比连体衣 / 娃丽比母婴旗舰店</t>
+          <t>嫚熙安睡裤 / EMXEE嫚熙母婴用品旗舰店</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>娃丽比连体衣 萌熊-N8 59cm</t>
+          <t>嫚熙安睡裤 XL码 4条×3包（共12条）</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>×3</t>
-        </is>
-      </c>
-      <c r="G55" s="2" t="inlineStr"/>
+          <t>×1</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="n">
+        <v>44.87</v>
+      </c>
       <c r="H55" s="2" t="n">
-        <v>199.76</v>
+        <v>35.9</v>
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>3316545230023087480</t>
+          <t>3316978813071005461</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>卖家已发货·申通</t>
+          <t>已付清·待发货</t>
         </is>
       </c>
       <c r="L55" s="2" t="inlineStr">
         <is>
-          <t>大牌59码连体衣</t>
+          <t>朋友清单未单列（同类品按需）</t>
         </is>
       </c>
       <c r="M55" s="2" t="inlineStr">
         <is>
-          <t>母婴A类；朋友张月推荐；性别中性；先洗后穿</t>
+          <t>已加购物车，未付款；大牌官方店/销量高</t>
         </is>
       </c>
       <c r="N55" s="2" t="inlineStr">
         <is>
-          <t>59合计：Baby love×3 + 娃丽比×3 = 6件；朋友推荐娃丽比≈¥70</t>
+          <t>大牌官方店替换小牌子（10-20）；商品 1077220832978</t>
         </is>
       </c>
       <c r="O55" s="2" t="inlineStr">
@@ -4291,14 +4293,14 @@
       <c r="C56" s="3" t="inlineStr"/>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>33单 54项</t>
+          <t>34单 54项</t>
         </is>
       </c>
       <c r="E56" s="3" t="inlineStr"/>
       <c r="F56" s="3" t="inlineStr"/>
       <c r="G56" s="3" t="inlineStr"/>
       <c r="H56" s="3" t="n">
-        <v>12934.56</v>
+        <v>12944.49</v>
       </c>
       <c r="I56" s="3" t="inlineStr"/>
       <c r="J56" s="3" t="inlineStr"/>
@@ -4319,7 +4321,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4441,7 +4443,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>已付清</t>
+          <t>已签收·韵达·3栋乙3号丰巢柜</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -4479,7 +4481,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>已付清</t>
+          <t>已签收·圆通·甲单元丰巢柜</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -4517,7 +4519,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>卖家已发货·中通</t>
+          <t>已签收·中通·家门口签收</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -4551,7 +4553,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>已付清</t>
+          <t>已签收·中通·3栋乙1号丰巢柜</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -4733,7 +4735,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>已付清</t>
+          <t>已签收·中通·3栋乙1号丰巢柜</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
@@ -4903,7 +4905,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>已付清</t>
+          <t>已签收·申通·3栋乙3号丰巢柜</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr"/>
@@ -4971,7 +4973,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>已付清</t>
+          <t>已签收·韵达·3栋乙3号丰巢柜</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr"/>
@@ -5039,7 +5041,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>已付清</t>
+          <t>已签收·家门口签收</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
@@ -5061,22 +5063,26 @@
         </is>
       </c>
       <c r="D21" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>嫚熙安睡裤 M-L 4条装（共8条）；嫚熙私处冲洗器 抗菌款</t>
+          <t>嫚熙私处冲洗器 抗菌款</t>
         </is>
       </c>
       <c r="F21" s="2" t="n">
-        <v>54.65</v>
+        <v>28.68</v>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>已付清</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr"/>
+          <t>已签收·中通·丰巢柜</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>原同单嫚熙安睡裤M-L×2包(¥25.97)因尺码偏小已退货退款(取件码6413)，已重拍XL码3包新单3316978813071005461</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -5107,7 +5113,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>已付清</t>
+          <t>已签收·申通·3栋乙3号丰巢柜</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr"/>
@@ -5277,7 +5283,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>卖家已发货·极兔</t>
+          <t>已签收·极兔·家门口签收</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -5311,7 +5317,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>已付清</t>
+          <t>已签收·中通·3栋乙1号丰巢柜</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr"/>
@@ -5413,7 +5419,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>已付清</t>
+          <t>已签收·圆通·3栋乙2号丰巢柜</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
@@ -5485,7 +5491,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>已付清</t>
+          <t>已签收·申通·3栋乙3号丰巢柜</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr"/>
@@ -5525,22 +5531,60 @@
       <c r="H34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>3316978813071005461</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>EMXEE嫚熙母婴用品旗舰店</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>嫚熙安睡裤 XL码 4条×3包（共12条）</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="n">
+        <v>35.9</v>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>已付清·待发货</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>替换原M-L码2包（孕20周身高160/体重120斤/臀围106cm，换XL加大码4条×3包共12条）</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>合计</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr"/>
-      <c r="C35" s="3" t="inlineStr"/>
-      <c r="D35" s="3" t="n">
+      <c r="B36" s="3" t="inlineStr"/>
+      <c r="C36" s="3" t="inlineStr"/>
+      <c r="D36" s="3" t="n">
         <v>54</v>
       </c>
-      <c r="E35" s="3" t="inlineStr"/>
-      <c r="F35" s="3" t="n">
-        <v>12934.5</v>
-      </c>
-      <c r="G35" s="3" t="inlineStr"/>
-      <c r="H35" s="3" t="inlineStr"/>
+      <c r="E36" s="3" t="inlineStr"/>
+      <c r="F36" s="3" t="n">
+        <v>12944.43</v>
+      </c>
+      <c r="G36" s="3" t="inlineStr"/>
+      <c r="H36" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>